<commit_message>
FIX: porgramas y creditos
</commit_message>
<xml_diff>
--- a/documentos/FCI & RESOLUCIONES 2025.xlsx
+++ b/documentos/FCI & RESOLUCIONES 2025.xlsx
@@ -16709,7 +16709,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2743"/>
+  <dimension ref="A1:Z2747"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.6640625" bestFit="1" customWidth="1" style="63" min="1" max="1"/>
@@ -66076,6 +66076,86 @@
         </is>
       </c>
     </row>
+    <row r="2744">
+      <c r="A2744" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="B2744" t="n">
+        <v>378</v>
+      </c>
+      <c r="C2744" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2744" t="inlineStr">
+        <is>
+          <t>Res. 378 Homologación Ingeniería de Sistemas y Telecomunicaciones JOHN JAIDER CARDONA TORO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2745">
+      <c r="A2745" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="B2745" t="n">
+        <v>379</v>
+      </c>
+      <c r="C2745" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2745" t="inlineStr">
+        <is>
+          <t>Res. 379 Homologación Ingeniería en Sistemas y Telecomunicaciones Presencial JUAN DAVID GÓMEZ VALLEJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2746">
+      <c r="A2746" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="B2746" t="n">
+        <v>380</v>
+      </c>
+      <c r="C2746" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2746" t="inlineStr">
+        <is>
+          <t>Res. 380 Homologación Ingeniería en Sistemas y Telecomunicaciones Presencial JUAN DAVID GÓMEZ VALLEJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2747">
+      <c r="A2747" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="B2747" t="n">
+        <v>381</v>
+      </c>
+      <c r="C2747" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2747" t="inlineStr">
+        <is>
+          <t>Res. 381 Homologación Ingeniería en Seguridad de la Información Presencial JUAN DAVID GÓMEZ VALLEJO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1042:D1042"/>

</xml_diff>

<commit_message>
FIX: colores FEATURE: homologaciones ESRI
</commit_message>
<xml_diff>
--- a/documentos/FCI & RESOLUCIONES 2025.xlsx
+++ b/documentos/FCI & RESOLUCIONES 2025.xlsx
@@ -16709,7 +16709,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2747"/>
+  <dimension ref="A1:Z2749"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.6640625" bestFit="1" customWidth="1" style="63" min="1" max="1"/>
@@ -66156,6 +66156,46 @@
         </is>
       </c>
     </row>
+    <row r="2748">
+      <c r="A2748" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="B2748" t="n">
+        <v>382</v>
+      </c>
+      <c r="C2748" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2748" t="inlineStr">
+        <is>
+          <t>Res. 382 Homologación Ingeniería Industrial PAULA HERNANDEZ MUÑOZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2749">
+      <c r="A2749" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="B2749" t="n">
+        <v>383</v>
+      </c>
+      <c r="C2749" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2749" t="inlineStr">
+        <is>
+          <t>Res. 383 Homologación Ingeniería en analítica de datos virtual PAULA HERNANDEZ MUÑOZ</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1042:D1042"/>

</xml_diff>

<commit_message>
FEATURE: codigo de asignaturas FIX: plantilla
</commit_message>
<xml_diff>
--- a/documentos/FCI & RESOLUCIONES 2025.xlsx
+++ b/documentos/FCI & RESOLUCIONES 2025.xlsx
@@ -16709,7 +16709,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2749"/>
+  <dimension ref="A1:Z2756"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.6640625" bestFit="1" customWidth="1" style="63" min="1" max="1"/>
@@ -66196,6 +66196,146 @@
         </is>
       </c>
     </row>
+    <row r="2750">
+      <c r="A2750" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="B2750" t="n">
+        <v>384</v>
+      </c>
+      <c r="C2750" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2750" t="inlineStr">
+        <is>
+          <t>Res. 384 Homologación Ingeniería en Sistemas y Telecomunicaciones Presencial JOHN JAIDER CARDONA TORO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2751">
+      <c r="A2751" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="B2751" t="n">
+        <v>385</v>
+      </c>
+      <c r="C2751" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2751" t="inlineStr">
+        <is>
+          <t>Res. 385 Homologación Ingeniería en analítica de datos virtual JOHN JAIDER CARDONA TORO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2752">
+      <c r="A2752" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="B2752" t="n">
+        <v>386</v>
+      </c>
+      <c r="C2752" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2752" t="inlineStr">
+        <is>
+          <t>Res. 386 Homologación Ingeniería en analítica de datos virtual JOHN JAIDER CARDONA TORO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2753">
+      <c r="A2753" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="B2753" t="n">
+        <v>387</v>
+      </c>
+      <c r="C2753" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2753" t="inlineStr">
+        <is>
+          <t>Res. 387 Homologación Ingeniería Logística Presencial JUAN DAVID GÓMEZ VALLEJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2754">
+      <c r="A2754" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="B2754" t="n">
+        <v>388</v>
+      </c>
+      <c r="C2754" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2754" t="inlineStr">
+        <is>
+          <t>Res. 388 Homologación Ingeniería en analítica de datos presencial JUAN DAVID GÓMEZ VALLEJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2755">
+      <c r="A2755" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="B2755" t="n">
+        <v>389</v>
+      </c>
+      <c r="C2755" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2755" t="inlineStr">
+        <is>
+          <t>Res. 389 Homologación Ingeniería Logística Presencial JOHN JAIDER CARDONA TORO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2756">
+      <c r="A2756" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="B2756" t="n">
+        <v>390</v>
+      </c>
+      <c r="C2756" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2756" t="inlineStr">
+        <is>
+          <t>Res. 390 Homologación Ingeniería Industrial CRISTIAN CAMILO SOTO JIMENEZ</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1042:D1042"/>

</xml_diff>

<commit_message>
FIX: notificaciones y validaciones en el formulario
</commit_message>
<xml_diff>
--- a/documentos/FCI & RESOLUCIONES 2025.xlsx
+++ b/documentos/FCI & RESOLUCIONES 2025.xlsx
@@ -16709,7 +16709,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2756"/>
+  <dimension ref="A1:Z2759"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.6640625" bestFit="1" customWidth="1" style="63" min="1" max="1"/>
@@ -66336,6 +66336,66 @@
         </is>
       </c>
     </row>
+    <row r="2757">
+      <c r="A2757" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="B2757" t="n">
+        <v>391</v>
+      </c>
+      <c r="C2757" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2757" t="inlineStr">
+        <is>
+          <t>Res. 391 Homologación Ingeniería en Sistemas y Telecomunicaciones Presencial JUAN DAVID GÓMEZ VALLEJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2758">
+      <c r="A2758" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="B2758" t="n">
+        <v>392</v>
+      </c>
+      <c r="C2758" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2758" t="inlineStr">
+        <is>
+          <t>Res. 392 Homologación Ingeniería Industrial PAULA HERNANDEZ MUÑOZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2759">
+      <c r="A2759" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="B2759" t="n">
+        <v>393</v>
+      </c>
+      <c r="C2759" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2759" t="inlineStr">
+        <is>
+          <t>Res. 393 Homologación Ingeniería en Sistemas y Telecomunicaciones Presencial JUAN DAVID GÓMEZ VALLEJO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1042:D1042"/>

</xml_diff>

<commit_message>
FIX: nombre de programas y cantidad de certificados por credito
</commit_message>
<xml_diff>
--- a/documentos/FCI & RESOLUCIONES 2025.xlsx
+++ b/documentos/FCI & RESOLUCIONES 2025.xlsx
@@ -16709,7 +16709,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2759"/>
+  <dimension ref="A1:Z2761"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.6640625" bestFit="1" customWidth="1" style="63" min="1" max="1"/>
@@ -66396,6 +66396,46 @@
         </is>
       </c>
     </row>
+    <row r="2760">
+      <c r="A2760" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
+        </is>
+      </c>
+      <c r="B2760" t="n">
+        <v>394</v>
+      </c>
+      <c r="C2760" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2760" t="inlineStr">
+        <is>
+          <t>Res. 394 Homologación Especialización en Sistemas de Información Geográfica (Presencial) JUAN GOMEZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2761">
+      <c r="A2761" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
+        </is>
+      </c>
+      <c r="B2761" t="n">
+        <v>395</v>
+      </c>
+      <c r="C2761" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2761" t="inlineStr">
+        <is>
+          <t>Res. 395 Homologación Ingeniería en Sistemas y Telecomunicaciones CRISTIAN CAMILO SOTO JIMENEZ</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1042:D1042"/>

</xml_diff>

<commit_message>
FIX: logica pregrados y posgrados con los proveedores de certificados
</commit_message>
<xml_diff>
--- a/documentos/FCI & RESOLUCIONES 2025.xlsx
+++ b/documentos/FCI & RESOLUCIONES 2025.xlsx
@@ -16709,7 +16709,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2761"/>
+  <dimension ref="A1:Z2763"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.6640625" bestFit="1" customWidth="1" style="63" min="1" max="1"/>
@@ -66436,6 +66436,46 @@
         </is>
       </c>
     </row>
+    <row r="2762">
+      <c r="A2762" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
+        </is>
+      </c>
+      <c r="B2762" t="n">
+        <v>396</v>
+      </c>
+      <c r="C2762" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2762" t="inlineStr">
+        <is>
+          <t>Res. 396 Homologación Ingeniería en Analítica de Datos (Presencial) JUAN GOMEZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2763">
+      <c r="A2763" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="B2763" t="n">
+        <v>397</v>
+      </c>
+      <c r="C2763" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2763" t="inlineStr">
+        <is>
+          <t>Res. 397 Homologación Especialización en Sistemas de Información Geográfica (Presencial) DIANA MILENA GIRALDO VALENCIA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1042:D1042"/>

</xml_diff>

<commit_message>
FEATURE: panel de control de usuarios y programas  FIX: validaciones de fecha y nota
</commit_message>
<xml_diff>
--- a/documentos/FCI & RESOLUCIONES 2025.xlsx
+++ b/documentos/FCI & RESOLUCIONES 2025.xlsx
@@ -16709,7 +16709,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2763"/>
+  <dimension ref="A1:Z2764"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.44140625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.6640625" bestFit="1" customWidth="1" style="63" min="1" max="1"/>
@@ -66476,6 +66476,26 @@
         </is>
       </c>
     </row>
+    <row r="2764">
+      <c r="A2764" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="B2764" t="n">
+        <v>398</v>
+      </c>
+      <c r="C2764" t="inlineStr">
+        <is>
+          <t>Juan David Gomez</t>
+        </is>
+      </c>
+      <c r="D2764" t="inlineStr">
+        <is>
+          <t>Res. 398 Homologación Ingeniería en Sistemas y Telecomunicaciones JUAN DAVID GOMEZ</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1042:D1042"/>

</xml_diff>